<commit_message>
restructuring the studying method
</commit_message>
<xml_diff>
--- a/TheorynCoding/Maintain Excel/Studying.xlsx
+++ b/TheorynCoding/Maintain Excel/Studying.xlsx
@@ -1,21 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="6" rupBuild="9302"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\RND\Java Practical\Eclipse Workspace\java-code-practice\TheorynCoding\Maintain Excel\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A61B1A08-74D1-474B-BAC7-A6EF7475B690}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="144525"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -25,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="12">
   <si>
     <t>File Studing</t>
   </si>
@@ -33,9 +27,6 @@
     <t>Status</t>
   </si>
   <si>
-    <t>In-progress</t>
-  </si>
-  <si>
     <t>Sr No</t>
   </si>
   <si>
@@ -64,15 +55,12 @@
   </si>
   <si>
     <t>TheorynCoding\BasicOPPCollection\Overall\Overall QA</t>
-  </si>
-  <si>
-    <t>TheorynCoding\BasicOPPCollection\Overall\Welcome_Java_Example_Internal_Working -1</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -202,7 +190,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin typeface="Calibri Light"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -237,7 +225,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -414,15 +402,15 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C10"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:C9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="1"/>
@@ -433,7 +421,7 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>0</v>
@@ -447,10 +435,10 @@
         <v>1</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -458,10 +446,10 @@
         <v>2</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -469,10 +457,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -480,10 +468,10 @@
         <v>4</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -491,10 +479,10 @@
         <v>5</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -502,10 +490,10 @@
         <v>6</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -513,10 +501,10 @@
         <v>7</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -524,26 +512,15 @@
         <v>8</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="2">
-        <v>9</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C10" xr:uid="{D6967C0E-D72A-4E25-AFDA-0A54DAE738DD}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C9 C2:C8">
       <formula1>"In-progress,Pending,Complete"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>